<commit_message>
updated excel sheet generator, and found an error in it when trying to update the field sample sheet
</commit_message>
<xml_diff>
--- a/static/auto_sheets/Field Samples Requirements.xlsx
+++ b/static/auto_sheets/Field Samples Requirements.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,7 +499,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sampling depth reference</t>
+          <t>Broad-Scale Environmental Context</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -512,36 +512,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>msl</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>local surface</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CGG_3_000002</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Point from where the depth measurement was taken</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sample storage address</t>
+          <t>Sample storage location</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -556,27 +536,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Address </t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>The exact address where the sample. If it's stored at geological museum then you can just write "GM".</t>
+          <t xml:space="preserve">If working half and archive half are stored different places, report two locations seperated by semi-colon and preceded by either A: or W: </t>
         </is>
       </c>
     </row>
@@ -625,12 +605,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Sample storage address</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -638,35 +618,41 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>-45.5347</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-45.5347</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-45.5347</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>decimal degrees, max 3 digits, max 8 decimal points (-180 to 180)</t>
+          <t xml:space="preserve">Address </t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>The geographical origin of the sample as defined by longitude. The values should be reported in decimal degrees as precise as possible (max. 8 decimal points).</t>
+          <t>The exact address where the sample. If it's stored at geological museum then you can just write "GM".</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sample storage location</t>
+          <t>Elevation (meters)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -674,41 +660,37 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
-        </is>
+      <c r="D7" t="n">
+        <v>37</v>
+      </c>
+      <c r="E7" t="n">
+        <v>37</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Number (decimal allowed)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">If working half and archive half are stored different places, report two locations seperated by semi-colon and preceded by either A: or W: </t>
+          <t>Vertical height above mean sea level. Specify as negative number if below mean sea level.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Environmental Medium</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -716,25 +698,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>61.1399</v>
-      </c>
-      <c r="E8" t="n">
-        <v>61.1399</v>
-      </c>
-      <c r="F8" t="n">
-        <v>61.1399</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>decimal degrees using WGS84 GPS Standard. Max 2 digits, max 8 decimal points (-90 to 90)</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>The geographical origin of the sample as defined by latitude.</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -781,91 +749,79 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Disposal date</t>
+          <t>Water depth (m)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+          <t>Decimal numbers or integers</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Report when the sample was disposed.</t>
+          <t>Depth below surface of water body, from where the sample was taken</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Storing date</t>
+          <t>Site Type</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Outcrop</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Cave</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Lake</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Report when the sample was stored in the specified storage location.</t>
+          <t>The type of site the sediment cores where taken. E.g. ocean, marine, freshwater, brackish, ice caves, caves. Please use ENVO ontology: http://environmentontology.org/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Local Environmental Context</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -875,166 +831,138 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Outcrop</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Cave</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Lake</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Outcrop, cave, lake, bog etc.</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Miscellaneous Sample Measurements or Observations</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">water content: 10 %; </t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>water content: 10 %;</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>water content: 10 %; porosity: 5 %</t>
-        </is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-45.5347</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+          <t>decimal degrees, max 3 digits, max 8 decimal points (-180 to 180)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Any relevant measurements/observations taken of the field sample. If multiple: seperate by semi-colon.</t>
+          <t>The geographical origin of the sample as defined by longitude. The values should be reported in decimal degrees as precise as possible (max. 8 decimal points).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Miscellaneous Environmental Measurements or Observations</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">temperature: 7 celcius; </t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">temperature: 7 celcius; </t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>temperature: 7 celcius; cloud cover: overcast;</t>
-        </is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="E14" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="F14" t="n">
+        <v>61.1399</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+          <t>decimal degrees using WGS84 GPS Standard. Max 2 digits, max 8 decimal points (-90 to 90)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Any other relevant environmental measurements/observations. If multiple: seperate by semi-colon.</t>
+          <t>The geographical origin of the sample as defined by latitude.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Height above mean sea level (meters)</t>
+          <t>Country/Ocean</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>37</v>
-      </c>
-      <c r="E15" t="n">
-        <v>37</v>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Greenland</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>37.5</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Number (decimal allowed)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Specify as negative number if below mean sea level.</t>
+          <t>The geographical origin of the sample as defined by the country or sea name. Country or sea names should be chosen from the INSDC country list (http://insdc.org/country.html), or the GAZ ontology (http://purl.bioontology.org/ontology/GAZ)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Age Estimate (ka)</t>
+          <t>QR Code</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>int4range</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1042,36 +970,20 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>[1, 105)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>[1, 105)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>[1, 105)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Restricted mathematical notation of the form [&lt;no&gt;, &lt;no&gt;). Meaning only use "[" as the opening bracket and ")" as the closing bracket (decimals not allowed).</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Not c14, just an estimate</t>
+          <t>An id for the physical QR code on the sample</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Period Estimate</t>
+          <t>Region/Province/State</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1084,37 +996,21 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Holocene</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Holocene</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Pleistocene</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Full names seperated by comma</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Link to images</t>
+          <t>Age Estimate (to, KABP)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1122,29 +1018,37 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>litter layer</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>canopy</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Link to any relevant images of the sample.</t>
+          <t>Report the entity or entities which are in the sample or specimen’s local vicinity and which you believe have significant causal influences on your sample or specimen. We recommend using EnvO terms which are of smaller spatial grain than your entry for env_broad_scale. Terms, such as anatomical sites, from other OBO Library ontologies which interoperate with EnvO (e.g. UBERON) are accepted in this field. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS. Multiple values allowed if seperated by semi-colon.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marine isotope stage estimate</t>
+          <t>Sampling depth estimation (bottom, cm)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1154,35 +1058,39 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>Soul</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>Ocean water</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>pond water</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Report the environmental material(s) immediately surrounding the sample or specimen at the time of sampling. We recommend using subclasses of "environmental material" (http://purl.obolibrary.org/obo/ENVO_00010483). EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS . Terms from other OBO ontologies are permissible as long as they reference mass/volume nouns (e.g. air, water, blood) and not discrete, countable entities (e.g. a tree, a leaf, a table top).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Correlation depth (top, cm)</t>
+          <t>Comment</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1190,27 +1098,15 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>10</v>
-      </c>
-      <c r="E20" t="n">
-        <v>200</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>300.3</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Numbers (decimals allowed)</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>The local core depth  that correlates with the  correlation depth (bottom) of the core immediately below.</t>
-        </is>
-      </c>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1245,12 +1141,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Correlation depth (bottom, cm)</t>
+          <t>Link to images</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1258,37 +1154,29 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>10</v>
-      </c>
-      <c r="E22" t="n">
-        <v>200</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>300.3</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Numbers (decimals allowed)</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>The local core depth that correlates with the  correlation depth (top) of the core immediately above.</t>
+          <t>Link to any relevant images of the sample.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sampling depth (interval, cm)</t>
+          <t>Miscellaneous Environmental Measurements or Observations</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>int4range</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1298,39 +1186,39 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>[10, 50)</t>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>[10, 20)</t>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[-10, -5)</t>
+          <t>temperature: 7 celcius; cloud cover: overcast;</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Restricted mathematical notation of the form [&lt;no&gt;, &lt;no&gt;). Meaning only use "[" as the opening bracket and ")" as the closing bracket (decimals not allowed).</t>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Depth measurement for interval type samples (such as core) </t>
+          <t>Any other relevant environmental measurements/observations. If multiple: seperate by semi-colon.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sampling depth (discrete, cm)</t>
+          <t>Miscellaneous Sample Measurements or Observations</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>double precision</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1338,37 +1226,41 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>10</v>
-      </c>
-      <c r="E24" t="n">
-        <v>200</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water content: 10 %; </t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>water content: 10 %;</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>300.3</t>
+          <t>water content: 10 %; porosity: 5 %</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Numbers (decimals allowed)</t>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Depth measurement for discrete type samples (such as tube)</t>
+          <t>Any relevant measurements/observations taken of the field sample. If multiple: seperate by semi-colon.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Running Project Title</t>
+          <t>Disposal date</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1378,39 +1270,39 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Traversing European Coastlines</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Arctic Canada</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Arctic Canada</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Referencing this google sheet: https://docs.google.com/spreadsheets/d/10TWDtKMug4yzOQUP7Q4APIoPNHQXCFX_RasijIgyCAA/edit?usp=sharing</t>
+          <t>Report when the sample was disposed.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Storing date</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1420,34 +1312,34 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Specify the grant that funds the project.</t>
+          <t>Report when the sample was stored in the specified storage location.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PI (KU ID)</t>
+          <t>Grant</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1462,34 +1354,34 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KU Id</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>KU id of the principal investigator responsible for the project.</t>
+          <t>Specify the grant that funds the project.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sample provider(s)</t>
+          <t>PI (KU ID)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1514,29 +1406,29 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>hlj234; glj523</t>
+          <t>hlj234</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KU Ids</t>
+          <t>KU Id</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Unique KU id(s) of the person(s) responsible for the sample extraction, seperated by semicolon if multiple.</t>
+          <t>KU id of the principal investigator responsible for the project.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sampling Date</t>
+          <t>Age Estimate (from, KABP)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1546,34 +1438,34 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>105</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>1105</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Date when the sampling occured.</t>
+          <t>Not precise, just an estimate. Remember to fill out the "from" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sampling site</t>
+          <t>Period Estimate</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1588,34 +1480,30 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>Holocene</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>Holocene</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>Pleistocene</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>If relevant. Otherwise leave blank.</t>
-        </is>
-      </c>
+          <t>Full names seperated by comma</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>City/Town/Location</t>
+          <t>Marine isotope stage estimate</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1630,34 +1518,30 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>5e</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>5e</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>5e</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>If relevant. Otherwise leave blank.</t>
-        </is>
-      </c>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Country/Ocean</t>
+          <t>Sediment type</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1672,35 +1556,39 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Greenland</t>
+          <t>Lacustrine</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Glaciofluvial</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Glaciofluvial</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Eg. Glacial, Lacustrine, Fluvial, Aeolian, Peat, Soil</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>QR Code</t>
+          <t>Sampling Date</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1708,25 +1596,41 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>An id for the physical QR code on the sample</t>
+          <t>Date when the sampling occured.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sediment type</t>
+          <t>Correlation depth (top, cm)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1734,43 +1638,37 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Lacustrine</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Glaciofluvial</t>
-        </is>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="n">
+        <v>200</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Glaciofluvial</t>
+          <t>300.3</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Numbers (decimals allowed)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Eg. Glacial, Lacustrine
-Fluvial, Aeolian,Peat
-Soil</t>
+          <t>The local core depth  that correlates with the  correlation depth (bottom) of the core immediately below.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Correlation depth (bottom, cm)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1778,15 +1676,367 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" t="n">
+        <v>200</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>The local core depth that correlates with the  correlation depth (top) of the core immediately above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sample provider(s)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>hlj234; glj523</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>KU Ids</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Unique KU id(s) of the person(s) responsible for the sample extraction, seperated by semicolon if multiple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sampling depth estimation (top, cm)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>-10</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Integers and minus sign</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Depth measurement as measured from the top of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sampling depth (discrete, cm)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>double precision</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" t="n">
+        <v>200</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Depth measurement for discrete type samples (such as tube). Only fill this out if your sample type is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Running Project Title</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Traversing European Coastlines</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Arctic Canada</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Arctic Canada</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
           <t>text and/or numbers</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Referencing this google sheet: https://docs.google.com/spreadsheets/d/10TWDtKMug4yzOQUP7Q4APIoPNHQXCFX_RasijIgyCAA/edit?usp=sharing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>City/Town/Lake/Location</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>If relevant. Otherwise leave blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sampling Site</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Any other geographic location identifier that might be relevant. If the sample was taken from a known archeological site for example. Otherwise leave blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>-10</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Integers and minus sign</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Depth measurement as measured from the bottom of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1105</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Not precise, just an estimate. Remember to fill out the "from" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The geographical origin of the sample as defined by the region/province/state. If relevant. Otherwise leave blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Report the major environmental system the sample or specimen came from. The system(s) identified should have a coarse spatial grain, to provide the general environmental context of where the sampling was done (e.g. in the desert or a rainforest). We recommend using subclasses of EnvO’s biome class:  http://purl.obolibrary.org/obo/ENVO_00000428. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>